<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-02 Les pommes de Chouchou
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-02.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-02.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut quatre pommes pour le saladier. Le panier coince la capuche du manteau bleu. Elle pose le panier, enfile le manteau, choisit les pommes. Une pomme roule. Elle la rattrape. Le manteau rentre au crochet. Les pommes brillent.</t>
+          <t>Une pièce tinte. Le panier d'osier tape une botte. Un éclat de liste brille au bord du papier. Chouchou veut quatre pommes pour le saladier, maintenant. Elle tire : la capuche du manteau bleu pince l'anse. Elle pose le panier, enfile le manteau. Au marché, la pomme jaune roule ; sa manche bouscule une caisse. Elle refuse de foncer, retrouve l'éclat, pose la quatrième. Le manteau clic au crochet. L'éclat brille près du blanc.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le panier d'osier attend près des bottes. Une liste dépasse du bord. Le papier est un peu froissé. Une pièce tinte dans la poche de maman. De la rue, une clochette de vélo passe. Ça sent la pierre encore humide. Le marché n'est pas loin. Chouchou, tu as vu le panier ? Oui. Il est près des bottes. En ce moment, Chouchou lève le panier. Son manteau bleu pend au crochet. Le tissu a une petite capuche. La capuche est coincée sous l'anse. Le panier ne vient pas. Il tient, maman ! Pose le panier un moment. On prend le manteau d'abord. Chouchou pose le panier près des bottes. Elle prend le manteau bleu. Elle glisse un bras, puis l'autre. La capuche tapote son dos. Tu as les boutons ? Un, deux, trois. Parfait. Maintenant le panier. On va chercher des pommes ? Oui. Quatre, pour le saladier. Maman ouvre la porte. Le vent est frais. Il sent un peu le pain. Ils marchent vers le marché. Chouchou tient une anse du panier. Tu as chaud dans le manteau ? Oui. J'ai chaud dedans. Au marché, les étals sont colorés. Les pommes brillent. Une pomme est rouge. Une autre est jaune. On en prend quatre ? Quatre pommes. Maman pose trois pommes dans le panier. La quatrième pomme jaune roule. Elle part vers le bord de l'étal. Elle part ! Tu peux la rattraper ? Chouchou avance la main. La pomme est lisse et froide. Elle la pose dans le panier. Je l'ai ! Merci. Le panier devient un peu lourd. Chouchou sent le sucré des fruits. C'est l'heure de rentrer. Oui. On rentre. Ils rentrent. L'entrée est calme. Chouchou retire le manteau bleu. Elle le raccroche au crochet. Le crochet fait un petit clic. Le manteau est à sa place. Elle pose le panier près des bottes. Les pommes tapotent le fond. Tu as fini de poser le panier ? Oui, maman. Les pommes sont dedans.</t>
+          <t>Une pièce tinte, dans une poche. C'est la poche de maman. Le panier d'osier tape une botte grise. Chouchou connaît cette entrée. Elle connaît les bottes, le crochet, la porte. Pourtant, un détail paraît nouveau. Un éclat de liste brille au bord du papier. Le papier froissé dépasse du panier. Un quatre est écrit, minuscule. De la rue, une clochette de vélo passe. L'air sent la pierre, humide. Dans la cuisine, le saladier blanc attend. Chouchou, tu as vu le panier ? Oui, maman. Il est près des bottes. Je veux les pommes, maintenant ! Quatre, pour le saladier. En ce moment, Chouchou saisit le panier. Son manteau bleu pend au crochet. Le tissu a une petite capuche. La capuche glisse sous l'anse. Le panier refuse de venir. Il tient, maman ! Elle tire plus fort, d'un coup. L'anse pince la capuche bleue. Rien ne bouge. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Maman s'accroupit à la même hauteur. Tu veux tirer, ou regarder ? Je veux les pommes. Chouchou tire une dernière fois. Le panier reste coincé.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le panier d'osier attend près des bottes. Une liste dépasse du bord. Le papier est un peu froissé. Une pièce tinte dans la poche de maman. De la rue, une clochette de vélo passe. Ça sent la pierre encore humide. Le marché n'est pas loin. Chouchou, tu as vu le panier ? Oui. Il est près des bottes. En ce moment, Chouchou lève le panier. Son manteau bleu pend au crochet. Le tissu a une petite capuche. La capuche est coincée sous l'anse. Le panier ne vient pas. Il tient, maman ! Pose le panier un moment. On prend le manteau d'abord. Chouchou pose le panier près des bottes. Elle prend le manteau bleu. Elle glisse un bras, puis l'autre. La capuche tapote son dos. Tu as les boutons ? Un, deux, trois. Parfait. Maintenant le panier. On va chercher des pommes ? Oui. Quatre, pour le saladier. Maman ouvre la porte. Le vent est frais. Il sent un peu le pain. Ils marchent vers le marché. Chouchou tient une anse du panier. Tu as chaud dans le manteau ? Oui. J'ai chaud dedans. Au marché, les étals sont colorés. Les pommes brillent. Une pomme est rouge. Une autre est jaune. On en prend quatre ? Quatre pommes. Maman pose trois pommes dans le panier. La quatrième pomme jaune roule. Elle part vers le bord de l'étal. Elle part ! Tu peux la rattraper ? Chouchou avance la main. La pomme est lisse et froide. Elle la pose dans le panier. Je l'ai ! Merci. Le panier devient un peu lourd. Chouchou sent le sucré des fruits. C'est l'heure de rentrer. Oui. On rentre. Ils rentrent. L'entrée est calme. Chouchou retire le manteau bleu. Elle le raccroche au crochet. Le crochet fait un petit clic. Le manteau est à sa place. Elle pose le panier près des bottes. Les pommes tapotent le fond. Tu as fini de poser le panier ? Oui, maman. Les pommes sont dedans.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une pièce tinte, dans une poche. C'est la poche de maman. Le panier d'osier tape une botte grise. Chouchou connaît cette entrée. Elle connaît les bottes, le crochet, la porte. Pourtant, un détail paraît nouveau. Un &lt;emphasis level="moderate"&gt;éclat de liste&lt;/emphasis&gt; brille au bord du papier. Le papier froissé dépasse du panier. Un quatre est écrit, minuscule. De la rue, une clochette de vélo passe. L'air sent la pierre, humide. Dans la cuisine, le saladier blanc attend. Chouchou, tu as vu le panier ? Oui, maman. Il est près des bottes. Je veux les pommes, maintenant ! Quatre, pour le saladier. En ce moment, Chouchou saisit le panier. Son manteau bleu pend au crochet. Le tissu a une petite capuche. La capuche glisse sous l'anse. Le panier refuse de venir. Il tient, maman ! Elle tire plus fort, d'un coup. L'anse pince la capuche bleue. Rien ne bouge. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Maman s'accroupit à la même hauteur. Tu veux tirer, ou regarder ? Je veux les pommes. Chouchou tire une dernière fois. Le panier reste coincé.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kenzo est dans l'entrée. Maman ouvre la porte. Avant de sortir, Kenzo prend le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Le manteau est bleu. Il glisse un bras, puis l'autre. Ils sortent. Le vent est frais. Au marché, Kenzo garde le manteau. Ils achètent des pommes. Maman dit : on rentre. Ils rentrent. Kenzo retire le manteau. Il le raccroche au crochet. Le manteau est à sa place. Maman dit : avant de sortir, le manteau. En rentrant, on le pose. [pause]</t>
+          <t>Une pièce tinte, dans une poche. C'est la poche de maman. Le panier d'osier tape une botte grise. Chouchou connaît cette entrée. Elle connaît les bottes, le crochet, la porte. Pourtant, un détail paraît nouveau. Un &lt;emphasis&gt;éclat de liste&lt;/emphasis&gt; brille au bord du papier. Le papier froissé dépasse du panier. Un quatre est écrit, minuscule. De la rue, une clochette de vélo passe. L'air sent la pierre, humide. Dans la cuisine, le saladier blanc attend. Chouchou, tu as vu le panier ? Oui, maman. Il est près des bottes. Je veux les pommes, maintenant ! Quatre, pour le saladier. En ce moment, Chouchou saisit le panier. Son manteau bleu pend au crochet. Le tissu a une petite capuche. La capuche glisse sous l'anse. Le panier refuse de venir. Il tient, maman ! Elle tire plus fort, d'un coup. L'anse pince la capuche bleue. Rien ne bouge. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Maman s'accroupit à la même hauteur. Tu veux tirer, ou regarder ? Je veux les pommes. Chouchou tire une dernière fois. Le panier reste coincé. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de liste</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,78 +1326,46 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_pommes_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le panier d'osier attend près des bottes.
-narrateur|Une liste dépasse du bord.
-narrateur|Le papier est un peu froissé.
-narrateur|Une pièce tinte dans la poche de maman.
+          <t>narrateur|Une pièce tinte, dans une poche.
+narrateur|C'est la poche de maman.
+narrateur|Le panier d'osier tape une botte grise.
+narrateur|Chouchou connaît cette entrée.
+narrateur|Elle connaît les bottes, le crochet, la porte.
+narrateur|Pourtant, un détail paraît nouveau.
+narrateur|Un éclat de liste brille au bord du papier.
+narrateur|Le papier froissé dépasse du panier.
+narrateur|Un quatre est écrit, minuscule.
 narrateur|De la rue, une clochette de vélo passe.
-narrateur|Ça sent la pierre encore humide.
-narrateur|Le marché n'est pas loin.
+narrateur|L'air sent la pierre, humide.
+narrateur|Dans la cuisine, le saladier blanc attend.
 maman|Chouchou, tu as vu le panier ?
-enfant-f|Oui.
+enfant-f|Oui, maman.
 enfant-f|Il est près des bottes.
-narrateur|En ce moment, Chouchou lève le panier.
+enfant-f|Je veux les pommes, maintenant !
+maman|Quatre, pour le saladier.
+narrateur|En ce moment, Chouchou saisit le panier.
 narrateur|Son manteau bleu pend au crochet.
 narrateur|Le tissu a une petite capuche.
-narrateur|La capuche est coincée sous l'anse.
-narrateur|Le panier ne vient pas.
+narrateur|La capuche glisse sous l'anse.
+narrateur|Le panier refuse de venir.
 enfant-f|Il tient, maman !
-maman|Pose le panier un moment.
-maman|On prend le manteau d'abord.
-narrateur|Chouchou pose le panier près des bottes.
-narrateur|Elle prend le manteau bleu.
-narrateur|Elle glisse un bras, puis l'autre.
-narrateur|La capuche tapote son dos.
-maman|Tu as les boutons ?
-enfant-f|Un, deux, trois.
-maman|Parfait.
-maman|Maintenant le panier.
-enfant-f|On va chercher des pommes ?
-maman|Oui.
-maman|Quatre, pour le saladier.
-narrateur|Maman ouvre la porte.
-narrateur|Le vent est frais.
-narrateur|Il sent un peu le pain.
-narrateur|Ils marchent vers le marché.
-narrateur|Chouchou tient une anse du panier.
-maman|Tu as chaud dans le manteau ?
-enfant-f|Oui.
-enfant-f|J'ai chaud dedans.
-narrateur|Au marché, les étals sont colorés.
-narrateur|Les pommes brillent.
-narrateur|Une pomme est rouge.
-narrateur|Une autre est jaune.
-maman|On en prend quatre ?
-enfant-f|Quatre pommes.
-narrateur|Maman pose trois pommes dans le panier.
-narrateur|La quatrième pomme jaune roule.
-narrateur|Elle part vers le bord de l'étal.
-enfant-f|Elle part !
-maman|Tu peux la rattraper ?
-narrateur|Chouchou avance la main.
-narrateur|La pomme est lisse et froide.
-narrateur|Elle la pose dans le panier.
-enfant-f|Je l'ai !
-maman|Merci.
-narrateur|Le panier devient un peu lourd.
-narrateur|Chouchou sent le sucré des fruits.
-maman|C'est l'heure de rentrer.
-enfant-f|Oui.
-enfant-f|On rentre.
-narrateur|Ils rentrent.
-narrateur|L'entrée est calme.
-narrateur|Chouchou retire le manteau bleu.
-narrateur|Elle le raccroche au crochet.
-narrateur|Le crochet fait un petit clic.
-narrateur|Le manteau est à sa place.
-narrateur|Elle pose le panier près des bottes.
-narrateur|Les pommes tapotent le fond.
-maman|Tu as fini de poser le panier ?
-enfant-f|Oui, maman.
-enfant-f|Les pommes sont dedans.</t>
+narrateur|Elle tire plus fort, d'un coup.
+narrateur|L'anse pince la capuche bleue.
+narrateur|Rien ne bouge.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu veux tirer, ou regarder ?
+enfant-f|Je veux les pommes.
+narrateur|Chouchou tire une dernière fois.
+narrateur|Le panier reste coincé.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1429,17 +1397,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Chouchou ?</t>
+          <t>Avant de sortir, Chouchou s'arrête près du crochet. Que prend-elle, pour le marché ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de sortir, que prend Chouchou ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Avant de sortir, Chouchou s'arrête près du &lt;emphasis level="moderate"&gt;crochet&lt;/emphasis&gt;. Que prend-elle, pour le marché ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Avant de &lt;emphasis&gt;sortir&lt;/emphasis&gt;, que prend Kenzo ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Avant de sortir, Chouchou s'arrête près du &lt;emphasis&gt;crochet&lt;/emphasis&gt;. Que prend-elle, pour le marché ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1502,7 +1470,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1510,10 +1478,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1528,38 +1496,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>sortir</t>
+          <t>crochet</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1568,28 +1536,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=près_du_crochet_avant_de_sortir; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de sortir, que prend Chouchou ?</t>
+          <t>narrateur|Avant de sortir, Chouchou s'arrête près du crochet.
+maman|Que prend-elle, pour le marché ?</t>
         </is>
       </c>
     </row>
@@ -1616,17 +1585,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a pris le manteau bleu. Elle l'a mis pour le marché. Elle a rattrapé la pomme jaune. En rentrant, elle a raccroché. Tu as pris le manteau pour sortir. Il attend près des bottes. Oui. Près du panier.</t>
+          <t>J'arrête de tirer. Elle pose le panier près des bottes. L'éclat de liste reste au bord. Le manteau, d'abord. Elle prend le manteau bleu. Elle glisse un bras, puis l'autre. La capuche tapote son dos. Tu as les boutons ? Un, deux, trois. Ils tiennent bien. Un bouton reste un peu de travers. Je le remets. Elle pousse le bouton dans sa fente. Chouchou reprend le panier d'osier. On va chercher les pommes ? Oui, quatre, pour le saladier. Maman ouvre la porte. Le vent est frais, sur les joues. Il sent un peu le pain. Ils marchent vers le marché. Chouchou tient une anse du panier. Tu as chaud, dans le manteau ? Oui. J'ai chaud dedans. Le tissu bleu tape contre sa hanche. Le papier froissé fait un petit bruit. Les pavés luisent, un peu humides.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a pris le manteau bleu. Elle l'a mis pour le marché. Elle a rattrapé la pomme jaune. En rentrant, elle a raccroché. Tu as pris le manteau pour sortir. Il attend près des bottes. Oui. Près du panier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'arrête de tirer. Elle pose le panier près des bottes. L'éclat de liste reste au bord. Le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt;, d'abord. Elle prend le manteau bleu. Elle glisse un bras, puis l'autre. La capuche tapote son dos. Tu as les boutons ? Un, deux, trois. Ils tiennent bien. Un bouton reste un peu de travers. Je le remets. Elle pousse le bouton dans sa fente. Chouchou reprend le panier d'osier. On va chercher les pommes ? Oui, quatre, pour le saladier. Maman ouvre la porte. Le vent est frais, sur les joues. Il sent un peu le pain. Ils marchent vers le marché. Chouchou tient une anse du panier. Tu as chaud, dans le manteau ? Oui. J'ai chaud dedans. Le tissu bleu tape contre sa hanche. Le papier froissé fait un petit bruit. Les pavés luisent, un peu humides.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kenzo a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt; pour sortir. En rentrant, il l'a raccroché. [pause]</t>
+          <t>J'arrête de tirer. Elle pose le panier près des bottes. L'éclat de liste reste au bord. Le &lt;emphasis&gt;manteau&lt;/emphasis&gt;, d'abord. Elle prend le manteau bleu. Elle glisse un bras, puis l'autre. La capuche tapote son dos. Tu as les boutons ? Un, deux, trois. Ils tiennent bien. Un bouton reste un peu de travers. Je le remets. Elle pousse le bouton dans sa fente. Chouchou reprend le panier d'osier. On va chercher les pommes ? Oui, quatre, pour le saladier. Maman ouvre la porte. Le vent est frais, sur les joues. Il sent un peu le pain. Ils marchent vers le marché. Chouchou tient une anse du panier. Tu as chaud, dans le manteau ? Oui. J'ai chaud dedans. Le tissu bleu tape contre sa hanche. Le papier froissé fait un petit bruit. Les pavés luisent, un peu humides. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1673,7 +1642,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1681,10 +1650,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1721,16 +1690,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1739,10 +1708,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.92</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1755,19 +1724,43 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=le_manteau_puis_le_panier; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a pris le manteau bleu.
-narrateur|Elle l'a mis pour le marché.
-narrateur|Elle a rattrapé la pomme jaune.
-narrateur|En rentrant, elle a raccroché.
-maman|Tu as pris le manteau pour sortir.
-enfant-f|Il attend près des bottes.
-maman|Oui.
-maman|Près du panier.</t>
+          <t>enfant-f|J'arrête de tirer.
+narrateur|Elle pose le panier près des bottes.
+narrateur|L'éclat de liste reste au bord.
+enfant-f|Le manteau, d'abord.
+narrateur|Elle prend le manteau bleu.
+narrateur|Elle glisse un bras, puis l'autre.
+narrateur|La capuche tapote son dos.
+maman|Tu as les boutons ?
+enfant-f|Un, deux, trois.
+maman|Ils tiennent bien.
+narrateur|Un bouton reste un peu de travers.
+enfant-f|Je le remets.
+narrateur|Elle pousse le bouton dans sa fente.
+narrateur|Chouchou reprend le panier d'osier.
+enfant-f|On va chercher les pommes ?
+maman|Oui, quatre, pour le saladier.
+narrateur|Maman ouvre la porte.
+narrateur|Le vent est frais, sur les joues.
+narrateur|Il sent un peu le pain.
+narrateur|Ils marchent vers le marché.
+narrateur|Chouchou tient une anse du panier.
+maman|Tu as chaud, dans le manteau ?
+enfant-f|Oui.
+enfant-f|J'ai chaud dedans.
+narrateur|Le tissu bleu tape contre sa hanche.
+narrateur|Le papier froissé fait un petit bruit.
+narrateur|Les pavés luisent, un peu humides.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,porte</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1787,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose les pommes sur la table. Elles roulent un tout petit peu. Elles sentent le marché. Tu veux les ranger dans le saladier ? Chouchou les pose une par une. Le saladier devient coloré. Chouchou touche le manteau au crochet. Le tissu est encore un peu frais. Les pommes sont prêtes. Moi aussi. Oui. Toi aussi.</t>
+          <t>Au marché, les étals sont colorés. Les pommes brillent sous le vent. Une pomme est rouge. Une autre est jaune, bien ronde. On en prend quatre ? Quatre pommes, maintenant ! Maman pose trois pommes dans le panier. La quatrième, jaune, roule. Elle part vers le bord de l'étal. Elle part ! Chouchou veut courir d'un coup. Sa manche bleue bouscule une caisse. La caisse penche, un peu. Oh. Le sourire ne revient pas. Elle s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le panier. L'éclat de liste est là. Celui du bord, dans l'entrée. Quatre, comme sur le papier. Tu veux la pomme jaune ? Celle qui brille. Elle avance la main, sans se presser. La pomme est lisse et froide. Elle la pose dans le panier. Je l'ai. Merci d'avoir regardé, Chouchou. Le panier devient un peu lourd. Chouchou sent le sucré des fruits. C'est l'heure de rentrer ? Oui, on rentre.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose les pommes sur la table. Elles roulent un tout petit peu. Elles sentent le marché. Tu veux les ranger dans le saladier ? Chouchou les pose une par une. Le saladier devient coloré. Chouchou touche le manteau au crochet. Le tissu est encore un peu frais. Les pommes sont prêtes. Moi aussi. Oui. Toi aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Au marché, les étals sont colorés. Les pommes brillent sous le vent. Une pomme est rouge. Une autre est jaune, bien ronde. On en prend quatre ? Quatre pommes, maintenant ! Maman pose trois pommes dans le panier. La quatrième, jaune, roule. Elle part vers le bord de l'étal. Elle part ! Chouchou veut courir d'un coup. Sa manche bleue bouscule une caisse. La caisse penche, un peu. Oh. Le sourire ne revient pas. Elle s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le panier. L'&lt;emphasis level="moderate"&gt;éclat de liste&lt;/emphasis&gt; est là. Celui du bord, dans l'entrée. Quatre, comme sur le papier. Tu veux la pomme jaune ? Celle qui brille. Elle avance la main, sans se presser. La pomme est lisse et froide. Elle la pose dans le panier. Je l'ai. Merci d'avoir regardé, Chouchou. Le panier devient un peu lourd. Chouchou sent le sucré des fruits. C'est l'heure de rentrer ? Oui, on rentre.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman pose les pommes. Kenzo touche le &lt;emphasis&gt;manteau&lt;/emphasis&gt; au crochet. [pause]</t>
+          <t>&lt;low-pitch&gt;Au marché, les étals sont colorés. Les pommes brillent sous le vent. Une pomme est rouge. Une autre est jaune, bien ronde. On en prend quatre ? Quatre pommes, maintenant ! Maman pose trois pommes dans le panier. La quatrième, jaune, roule. Elle part vers le bord de l'étal. Elle part ! Chouchou veut courir d'un coup. Sa manche bleue bouscule une caisse. La caisse penche, un peu. Oh. Le sourire ne revient pas. Elle s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le panier. L'&lt;emphasis&gt;éclat de liste&lt;/emphasis&gt; est là. Celui du bord, dans l'entrée. Quatre, comme sur le papier. Tu veux la pomme jaune ? Celle qui brille. Elle avance la main, sans se presser. La pomme est lisse et froide. Elle la pose dans le panier. Je l'ai. Merci d'avoir regardé, Chouchou. Le panier devient un peu lourd. Chouchou sent le sucré des fruits. C'est l'heure de rentrer ? Oui, on rentre.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1851,7 +1844,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1859,22 +1852,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1885,30 +1882,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de liste</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1917,35 +1914,65 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_éclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman pose les pommes sur la table.
-narrateur|Elles roulent un tout petit peu.
-enfant-f|Elles sentent le marché.
-maman|Tu veux les ranger dans le saladier ?
-narrateur|Chouchou les pose une par une.
-narrateur|Le saladier devient coloré.
-narrateur|Chouchou touche le manteau au crochet.
-narrateur|Le tissu est encore un peu frais.
-maman|Les pommes sont prêtes.
-enfant-f|Moi aussi.
-maman|Oui.
-maman|Toi aussi.</t>
+          <t>narrateur|Au marché, les étals sont colorés.
+narrateur|Les pommes brillent sous le vent.
+narrateur|Une pomme est rouge.
+narrateur|Une autre est jaune, bien ronde.
+maman|On en prend quatre ?
+enfant-f|Quatre pommes, maintenant !
+narrateur|Maman pose trois pommes dans le panier.
+narrateur|La quatrième, jaune, roule.
+narrateur|Elle part vers le bord de l'étal.
+enfant-f|Elle part !
+narrateur|Chouchou veut courir d'un coup.
+narrateur|Sa manche bleue bouscule une caisse.
+narrateur|La caisse penche, un peu.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Elle s'arrête net.
+enfant-f|Pas maintenant.
+narrateur|Elle refuse de foncer.
+narrateur|Elle lève les yeux vers le panier.
+narrateur|L'éclat de liste est là.
+narrateur|Celui du bord, dans l'entrée.
+enfant-f|Quatre, comme sur le papier.
+maman|Tu veux la pomme jaune ?
+enfant-f|Celle qui brille.
+narrateur|Elle avance la main, sans se presser.
+narrateur|La pomme est lisse et froide.
+narrateur|Elle la pose dans le panier.
+enfant-f|Je l'ai.
+maman|Merci d'avoir regardé, Chouchou.
+narrateur|Le panier devient un peu lourd.
+narrateur|Chouchou sent le sucré des fruits.
+maman|C'est l'heure de rentrer ?
+enfant-f|Oui, on rentre.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>marche,pomme</t>
         </is>
       </c>
     </row>
@@ -1972,17 +1999,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai mis les pommes dans le saladier. J'avais le manteau pour le marché. Bravo, Chouchou. Les pommes brillent dans le saladier.</t>
+          <t>Ils rentrent. L'entrée sent la pierre, froide. Chouchou retire le manteau bleu. Elle le raccroche au crochet. Le crochet fait un petit clic. Le manteau est à sa place. Elle pose le panier près des bottes. Les pommes tapotent le fond. Tu as fini de poser le panier ? Oui, maman. Les pommes sont dedans. Maman pose les pommes sur la table. Elles roulent un tout petit peu. Elles sentent le marché. Tu veux les mettre dans le saladier ? Chouchou les pose une par une. Le saladier devient coloré. L'éclat de liste brille près du blanc. Il est venu avec nous. Tu l'as vu, toi ? Il m'a montré les quatre. Le manteau bleu attend au crochet. Le saladier garde les quatre pommes.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai mis les pommes dans le saladier. J'avais le manteau pour le marché. Bravo, Chouchou. Les pommes brillent dans le saladier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent. L'entrée sent la pierre, froide. Chouchou retire le manteau bleu. Elle le raccroche au crochet. Le crochet fait un petit clic. Le manteau est à sa place. Elle pose le panier près des bottes. Les pommes tapotent le fond. Tu as fini de poser le panier ? Oui, maman. Les pommes sont dedans. Maman pose les pommes sur la table. Elles roulent un tout petit peu. Elles sentent le marché. Tu veux les mettre dans le saladier ? Chouchou les pose une par une. Le saladier devient coloré. L'&lt;emphasis level="moderate"&gt;éclat de liste&lt;/emphasis&gt; brille près du blanc. Il est venu avec nous. Tu l'as vu, toi ? Il m'a montré les quatre. Le manteau bleu attend au crochet. Le saladier garde les quatre pommes.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent. L'entrée sent la pierre, froide. Chouchou retire le manteau bleu. Elle le raccroche au crochet. Le crochet fait un petit clic. Le manteau est à sa place. Elle pose le panier près des bottes. Les pommes tapotent le fond. Tu as fini de poser le panier ? Oui, maman. Les pommes sont dedans. Maman pose les pommes sur la table. Elles roulent un tout petit peu. Elles sentent le marché. Tu veux les mettre dans le saladier ? Chouchou les pose une par une. Le saladier devient coloré. L'&lt;emphasis&gt;éclat de liste&lt;/emphasis&gt; brille près du blanc. Il est venu avec nous. Tu l'as vu, toi ? Il m'a montré les quatre. Le manteau bleu attend au crochet. Le saladier garde les quatre pommes.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2029,15 +2056,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2049,12 +2076,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2063,17 +2090,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de liste</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2082,11 +2113,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2095,27 +2126,55 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_du_bord_brille_près_du_saladier; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai mis les pommes dans le saladier.
-enfant-f|J'avais le manteau pour le marché.
-maman|Bravo, Chouchou.
-narrateur|Les pommes brillent dans le saladier.</t>
+          <t>narrateur|Ils rentrent.
+narrateur|L'entrée sent la pierre, froide.
+narrateur|Chouchou retire le manteau bleu.
+narrateur|Elle le raccroche au crochet.
+narrateur|Le crochet fait un petit clic.
+narrateur|Le manteau est à sa place.
+narrateur|Elle pose le panier près des bottes.
+narrateur|Les pommes tapotent le fond.
+maman|Tu as fini de poser le panier ?
+enfant-f|Oui, maman.
+enfant-f|Les pommes sont dedans.
+narrateur|Maman pose les pommes sur la table.
+narrateur|Elles roulent un tout petit peu.
+enfant-f|Elles sentent le marché.
+maman|Tu veux les mettre dans le saladier ?
+narrateur|Chouchou les pose une par une.
+narrateur|Le saladier devient coloré.
+narrateur|L'éclat de liste brille près du blanc.
+enfant-f|Il est venu avec nous.
+maman|Tu l'as vu, toi ?
+enfant-f|Il m'a montré les quatre.
+narrateur|Le manteau bleu attend au crochet.
+narrateur|Le saladier garde les quatre pommes.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>crochet,porte</t>
         </is>
       </c>
     </row>
@@ -2136,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2228,6 +2287,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>